<commit_message>
Refresh web app styling for professional light theme
</commit_message>
<xml_diff>
--- a/ornek-veriler/iSEM - LGS - 1 Detaylı Cevap Anahtarı.xlsx
+++ b/ornek-veriler/iSEM - LGS - 1 Detaylı Cevap Anahtarı.xlsx
@@ -1,37 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <bookViews>
+    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
+  </bookViews>
   <sheets>
-    <sheet name="Detaylı Cevap Anahtarı" sheetId="1" r:id="rId1"/>
+    <sheet name="Detaylı Cevap Anahtarı" sheetId="1" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="72">
   <si>
     <t>BÖLÜM</t>
   </si>
@@ -66,7 +46,7 @@
     <t>SÖZCÜKTE ANLAM</t>
   </si>
   <si>
-    <t>LGS TÜRKÇE</t>
+    <t>Türkçe</t>
   </si>
   <si>
     <t>19</t>
@@ -186,7 +166,7 @@
     <t>BİR KAHRAMAN DOĞUYOR</t>
   </si>
   <si>
-    <t>LGS T.C. İNKILAP TARİHİ VE ATATÜRKÇÜLÜK</t>
+    <t>Sosyal Bilgiler</t>
   </si>
   <si>
     <t>M. KEMAL'İN FİKİR HAYATINI ETKİLEYEN YERLER, OLAY VE KİŞİLER</t>
@@ -201,7 +181,7 @@
     <t>KAZA VE KADER</t>
   </si>
   <si>
-    <t>LGS DİN KÜLTÜRÜ VE AHLAK BİLGİSİ</t>
+    <t>Din Kültürü</t>
   </si>
   <si>
     <t>İNSAN İRADESİ VE KADER</t>
@@ -213,7 +193,7 @@
     <t>FRIENDSHIP</t>
   </si>
   <si>
-    <t>LGS İNGİLİZCE</t>
+    <t>İngilizce</t>
   </si>
   <si>
     <t>MATEMATİK</t>
@@ -225,7 +205,7 @@
     <t>ÇARPANLAR VE KATLAR</t>
   </si>
   <si>
-    <t>LGS MATEMATİK</t>
+    <t>Matematik</t>
   </si>
   <si>
     <t>NEGATİF KUVVET</t>
@@ -246,23 +226,31 @@
     <t>MEVSİMLER VE İKLİM</t>
   </si>
   <si>
-    <t>LGS FEN BİLİMLERİ</t>
+    <t>Fen Bilimleri</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="0" formatCode="General"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <sz val="12"/>
-      <color theme="1"/>
+      <color indexed="8"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color indexed="8"/>
+      <name val="Helvetica Neue"/>
+    </font>
+    <font>
+      <sz val="15"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -273,7 +261,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -281,36 +269,78 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="9"/>
+      </left>
+      <right style="thin">
+        <color indexed="9"/>
+      </right>
+      <top style="thin">
+        <color indexed="9"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="ff000000"/>
+      <rgbColor rgb="ffffffff"/>
+      <rgbColor rgb="ffff0000"/>
+      <rgbColor rgb="ff00ff00"/>
+      <rgbColor rgb="ff0000ff"/>
+      <rgbColor rgb="ffffff00"/>
+      <rgbColor rgb="ffff00ff"/>
+      <rgbColor rgb="ff00ffff"/>
+      <rgbColor rgb="ff000000"/>
+      <rgbColor rgb="ffaaaaaa"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office Theme">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="A7A7A7"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="535353"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="4F81BD"/>
@@ -334,82 +364,22 @@
         <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="FF00FF"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office Theme">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:latin typeface="Helvetica Neue"/>
+        <a:ea typeface="Helvetica Neue"/>
+        <a:cs typeface="Helvetica Neue"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:latin typeface="Helvetica Neue"/>
+        <a:ea typeface="Helvetica Neue"/>
+        <a:cs typeface="Helvetica Neue"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office Theme">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -443,7 +413,7 @@
               <a:schemeClr val="phClr">
                 <a:tint val="100000"/>
                 <a:shade val="100000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="129999"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
@@ -462,7 +432,7 @@
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
-              <a:satMod val="105000"/>
+              <a:satMod val="104999"/>
             </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
@@ -483,16 +453,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -501,23 +462,21 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="20000" dir="5400000">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -574,2148 +533,2964 @@
   </a:themeElements>
   <a:objectDefaults>
     <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
+      <a:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="25400" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:round/>
+        </a:ln>
+        <a:effectLst>
+          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
+            <a:srgbClr val="000000">
+              <a:alpha val="35000"/>
+            </a:srgbClr>
+          </a:outerShdw>
+        </a:effectLst>
+        <a:sp3d/>
+      </a:spPr>
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+        <a:spAutoFit/>
+      </a:bodyPr>
+      <a:lstStyle>
+        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+            <a:latin typeface="Calibri"/>
+            <a:ea typeface="Calibri"/>
+            <a:cs typeface="Calibri"/>
+            <a:sym typeface="Calibri"/>
+          </a:defRPr>
+        </a:defPPr>
+        <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl1pPr>
+        <a:lvl2pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl2pPr>
+        <a:lvl3pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl3pPr>
+        <a:lvl4pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl4pPr>
+        <a:lvl5pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl5pPr>
+        <a:lvl6pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl6pPr>
+        <a:lvl7pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl7pPr>
+        <a:lvl8pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl8pPr>
+        <a:lvl9pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl9pPr>
+      </a:lstStyle>
       <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="none"/>
       </a:style>
     </a:spDef>
     <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
+      <a:spPr>
+        <a:noFill/>
+        <a:ln w="25400" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:round/>
+        </a:ln>
+        <a:effectLst>
+          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="20000" dir="5400000">
+            <a:srgbClr val="000000">
+              <a:alpha val="38000"/>
+            </a:srgbClr>
+          </a:outerShdw>
+        </a:effectLst>
+        <a:sp3d/>
+      </a:spPr>
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+        <a:noAutofit/>
+      </a:bodyPr>
+      <a:lstStyle>
+        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:defPPr>
+        <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl1pPr>
+        <a:lvl2pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl2pPr>
+        <a:lvl3pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl3pPr>
+        <a:lvl4pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl4pPr>
+        <a:lvl5pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl5pPr>
+        <a:lvl6pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl6pPr>
+        <a:lvl7pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl7pPr>
+        <a:lvl8pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl8pPr>
+        <a:lvl9pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl9pPr>
+      </a:lstStyle>
       <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="none"/>
       </a:style>
     </a:lnDef>
+    <a:txDef>
+      <a:spPr>
+        <a:noFill/>
+        <a:ln w="12700" cap="flat">
+          <a:noFill/>
+          <a:miter lim="400000"/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </a:spPr>
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+        <a:spAutoFit/>
+      </a:bodyPr>
+      <a:lstStyle>
+        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+            <a:latin typeface="Calibri"/>
+            <a:ea typeface="Calibri"/>
+            <a:cs typeface="Calibri"/>
+            <a:sym typeface="Calibri"/>
+          </a:defRPr>
+        </a:defPPr>
+        <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl1pPr>
+        <a:lvl2pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl2pPr>
+        <a:lvl3pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl3pPr>
+        <a:lvl4pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl4pPr>
+        <a:lvl5pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl5pPr>
+        <a:lvl6pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl6pPr>
+        <a:lvl7pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl7pPr>
+        <a:lvl8pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl8pPr>
+        <a:lvl9pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
+          <a:lnSpc>
+            <a:spcPct val="100000"/>
+          </a:lnSpc>
+          <a:spcBef>
+            <a:spcPts val="0"/>
+          </a:spcBef>
+          <a:spcAft>
+            <a:spcPts val="0"/>
+          </a:spcAft>
+          <a:buClrTx/>
+          <a:buSzTx/>
+          <a:buFontTx/>
+          <a:buNone/>
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:uFillTx/>
+          </a:defRPr>
+        </a:lvl9pPr>
+      </a:lstStyle>
+      <a:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="none"/>
+      </a:style>
+    </a:txDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:G91"/>
+  <sheetFormatPr defaultColWidth="8" defaultRowHeight="12.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="6" width="8" style="1" customWidth="1"/>
+    <col min="7" max="7" width="51.4453" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8" style="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
+    <row r="1" ht="15.35" customHeight="1">
+      <c r="A1" t="s" s="2">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="2">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="2">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="2">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="2">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="2">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s">
+    <row r="2" ht="15.35" customHeight="1">
+      <c r="A2" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="3">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="2">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" t="s" s="2">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="2">
         <v>10</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="s">
+    <row r="3" ht="15.35" customHeight="1">
+      <c r="A3" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="3">
         <v>2</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" t="s" s="2">
         <v>12</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="s">
+    <row r="4" ht="15.35" customHeight="1">
+      <c r="A4" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="3">
         <v>3</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" t="s" s="2">
         <v>15</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="s">
+    <row r="5" ht="15.35" customHeight="1">
+      <c r="A5" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="3">
         <v>4</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" t="s" s="2">
         <v>17</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" t="s" s="2">
         <v>18</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" t="s" s="2">
         <v>19</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="s">
+    <row r="6" ht="15.35" customHeight="1">
+      <c r="A6" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="3">
         <v>5</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" t="s" s="2">
         <v>21</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" t="s" s="2">
         <v>10</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="s">
+    <row r="7" ht="15.35" customHeight="1">
+      <c r="A7" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="3">
         <v>6</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" t="s" s="2">
         <v>10</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" t="s" s="2">
         <v>10</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="s">
+    <row r="8" ht="15.35" customHeight="1">
+      <c r="A8" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="3">
         <v>7</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" t="s" s="2">
         <v>18</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" t="s" s="2">
         <v>19</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="s">
+    <row r="9" ht="15.35" customHeight="1">
+      <c r="A9" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="3">
         <v>8</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="s">
+    <row r="10" ht="15.35" customHeight="1">
+      <c r="A10" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="3">
         <v>9</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" t="s" s="2">
         <v>27</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="s">
+    <row r="11" ht="15.35" customHeight="1">
+      <c r="A11" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="3">
         <v>10</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" t="s" s="2">
         <v>28</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="s">
+    <row r="12" ht="15.35" customHeight="1">
+      <c r="A12" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="3">
         <v>11</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" t="s" s="2">
         <v>29</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" t="s" s="2">
         <v>30</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" t="s" s="2">
         <v>30</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="s">
+    <row r="13" ht="15.35" customHeight="1">
+      <c r="A13" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="3">
         <v>12</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" t="s" s="2">
         <v>31</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="s">
+    <row r="14" ht="15.35" customHeight="1">
+      <c r="A14" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="3">
         <v>13</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" t="s" s="2">
         <v>32</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="s">
+    <row r="15" ht="15.35" customHeight="1">
+      <c r="A15" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="3">
         <v>14</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" t="s" s="2">
         <v>33</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" t="s" s="2">
         <v>34</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" t="s" s="2">
         <v>35</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="s">
+    <row r="16" ht="15.35" customHeight="1">
+      <c r="A16" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="3">
         <v>15</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" t="s" s="2">
         <v>36</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" t="s" s="2">
         <v>37</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="s">
+    <row r="17" ht="15.35" customHeight="1">
+      <c r="A17" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="3">
         <v>16</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" t="s" s="2">
         <v>39</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="s">
+    <row r="18" ht="15.35" customHeight="1">
+      <c r="A18" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="3">
         <v>17</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" t="s" s="2">
         <v>40</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G18" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="s">
+    <row r="19" ht="15.35" customHeight="1">
+      <c r="A19" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="3">
         <v>18</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" t="s" s="2">
         <v>42</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" t="s" s="2">
         <v>42</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G19" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="s">
+    <row r="20" ht="15.35" customHeight="1">
+      <c r="A20" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="3">
         <v>19</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" t="s" s="2">
         <v>43</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" t="s" s="2">
         <v>44</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" t="s" s="2">
         <v>45</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G20" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="s">
+    <row r="21" ht="15.35" customHeight="1">
+      <c r="A21" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="3">
         <v>20</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" t="s" s="2">
         <v>46</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" t="s" s="2">
         <v>47</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" t="s" s="2">
         <v>45</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G21" t="s" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="s">
+    <row r="22" ht="15.35" customHeight="1">
+      <c r="A22" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="3">
         <v>1</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" t="s" s="2">
         <v>29</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" t="s" s="2">
         <v>49</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G22" t="s" s="2">
         <v>51</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="s">
+    <row r="23" ht="15.35" customHeight="1">
+      <c r="A23" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="3">
         <v>2</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" t="s" s="2">
         <v>31</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" t="s" s="2">
         <v>49</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="2">
         <v>51</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="s">
+    <row r="24" ht="15.35" customHeight="1">
+      <c r="A24" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="3">
         <v>3</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" t="s" s="2">
         <v>32</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" t="s" s="2">
         <v>52</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="G24" t="s">
+      <c r="G24" t="s" s="2">
         <v>51</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="s">
+    <row r="25" ht="15.35" customHeight="1">
+      <c r="A25" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="3">
         <v>4</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" t="s" s="2">
         <v>33</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" t="s" s="2">
         <v>53</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25" t="s" s="2">
         <v>51</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="s">
+    <row r="26" ht="15.35" customHeight="1">
+      <c r="A26" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="3">
         <v>5</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" t="s" s="2">
         <v>36</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" t="s" s="2">
         <v>53</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F26" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G26" t="s" s="2">
         <v>51</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="s">
+    <row r="27" ht="15.35" customHeight="1">
+      <c r="A27" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="3">
         <v>6</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" t="s" s="2">
         <v>49</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="G27" t="s">
+      <c r="G27" t="s" s="2">
         <v>51</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="s">
+    <row r="28" ht="15.35" customHeight="1">
+      <c r="A28" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="3">
         <v>7</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" t="s" s="2">
         <v>40</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E28" t="s" s="2">
         <v>53</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F28" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="G28" t="s">
+      <c r="G28" t="s" s="2">
         <v>51</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="s">
+    <row r="29" ht="15.35" customHeight="1">
+      <c r="A29" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="B29">
+      <c r="B29" s="3">
         <v>8</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E29" t="s" s="2">
         <v>49</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F29" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="G29" t="s">
+      <c r="G29" t="s" s="2">
         <v>51</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="s">
+    <row r="30" ht="15.35" customHeight="1">
+      <c r="A30" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="B30">
+      <c r="B30" s="3">
         <v>9</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" t="s" s="2">
         <v>43</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" t="s" s="2">
         <v>52</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="G30" t="s">
+      <c r="G30" t="s" s="2">
         <v>51</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="s">
+    <row r="31" ht="15.35" customHeight="1">
+      <c r="A31" t="s" s="2">
         <v>48</v>
       </c>
-      <c r="B31">
+      <c r="B31" s="3">
         <v>10</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" t="s" s="2">
         <v>46</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" t="s" s="2">
         <v>53</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31" t="s" s="2">
         <v>50</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G31" t="s" s="2">
         <v>51</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="s">
+    <row r="32" ht="15.35" customHeight="1">
+      <c r="A32" t="s" s="2">
         <v>54</v>
       </c>
-      <c r="B32">
+      <c r="B32" s="3">
         <v>1</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" t="s" s="2">
         <v>29</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E32" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F32" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G32" t="s" s="2">
         <v>56</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="s">
+    <row r="33" ht="15.35" customHeight="1">
+      <c r="A33" t="s" s="2">
         <v>54</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="3">
         <v>2</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" t="s" s="2">
         <v>31</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E33" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F33" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="G33" t="s">
+      <c r="G33" t="s" s="2">
         <v>56</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="s">
+    <row r="34" ht="15.35" customHeight="1">
+      <c r="A34" t="s" s="2">
         <v>54</v>
       </c>
-      <c r="B34">
+      <c r="B34" s="3">
         <v>3</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C34" t="s" s="2">
         <v>32</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E34" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F34" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="G34" t="s">
+      <c r="G34" t="s" s="2">
         <v>56</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="s">
+    <row r="35" ht="15.35" customHeight="1">
+      <c r="A35" t="s" s="2">
         <v>54</v>
       </c>
-      <c r="B35">
+      <c r="B35" s="3">
         <v>4</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" t="s" s="2">
         <v>33</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E35" t="s">
+      <c r="E35" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F35" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="G35" t="s">
+      <c r="G35" t="s" s="2">
         <v>56</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="s">
+    <row r="36" ht="15.35" customHeight="1">
+      <c r="A36" t="s" s="2">
         <v>54</v>
       </c>
-      <c r="B36">
+      <c r="B36" s="3">
         <v>5</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C36" t="s" s="2">
         <v>36</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D36" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E36" t="s">
+      <c r="E36" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="F36" t="s">
+      <c r="F36" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="G36" t="s">
+      <c r="G36" t="s" s="2">
         <v>56</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="s">
+    <row r="37" ht="15.35" customHeight="1">
+      <c r="A37" t="s" s="2">
         <v>54</v>
       </c>
-      <c r="B37">
+      <c r="B37" s="3">
         <v>6</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C37" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D37" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E37" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="F37" t="s">
+      <c r="F37" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="G37" t="s">
+      <c r="G37" t="s" s="2">
         <v>56</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="s">
+    <row r="38" ht="15.35" customHeight="1">
+      <c r="A38" t="s" s="2">
         <v>54</v>
       </c>
-      <c r="B38">
+      <c r="B38" s="3">
         <v>7</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C38" t="s" s="2">
         <v>40</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E38" t="s">
+      <c r="E38" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="F38" t="s">
+      <c r="F38" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="G38" t="s">
+      <c r="G38" t="s" s="2">
         <v>56</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="s">
+    <row r="39" ht="15.35" customHeight="1">
+      <c r="A39" t="s" s="2">
         <v>54</v>
       </c>
-      <c r="B39">
+      <c r="B39" s="3">
         <v>8</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C39" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D39" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E39" t="s">
+      <c r="E39" t="s" s="2">
         <v>57</v>
       </c>
-      <c r="F39" t="s">
+      <c r="F39" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="G39" t="s">
+      <c r="G39" t="s" s="2">
         <v>56</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="s">
+    <row r="40" ht="15.35" customHeight="1">
+      <c r="A40" t="s" s="2">
         <v>54</v>
       </c>
-      <c r="B40">
+      <c r="B40" s="3">
         <v>9</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C40" t="s" s="2">
         <v>43</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D40" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E40" t="s">
+      <c r="E40" t="s" s="2">
         <v>57</v>
       </c>
-      <c r="F40" t="s">
+      <c r="F40" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="G40" t="s">
+      <c r="G40" t="s" s="2">
         <v>56</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="s">
+    <row r="41" ht="15.35" customHeight="1">
+      <c r="A41" t="s" s="2">
         <v>54</v>
       </c>
-      <c r="B41">
+      <c r="B41" s="3">
         <v>10</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C41" t="s" s="2">
         <v>46</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D41" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E41" t="s">
+      <c r="E41" t="s" s="2">
         <v>57</v>
       </c>
-      <c r="F41" t="s">
+      <c r="F41" t="s" s="2">
         <v>55</v>
       </c>
-      <c r="G41" t="s">
+      <c r="G41" t="s" s="2">
         <v>56</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="s">
+    <row r="42" ht="15.35" customHeight="1">
+      <c r="A42" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="B42">
+      <c r="B42" s="3">
         <v>1</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C42" t="s" s="2">
         <v>29</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D42" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E42" t="s">
+      <c r="E42" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="F42" t="s">
+      <c r="F42" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="G42" t="s">
+      <c r="G42" t="s" s="2">
         <v>60</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="s">
+    <row r="43" ht="15.35" customHeight="1">
+      <c r="A43" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="B43">
+      <c r="B43" s="3">
         <v>2</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C43" t="s" s="2">
         <v>31</v>
       </c>
-      <c r="D43" t="s">
+      <c r="D43" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E43" t="s">
+      <c r="E43" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="F43" t="s">
+      <c r="F43" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="G43" t="s">
+      <c r="G43" t="s" s="2">
         <v>60</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="s">
+    <row r="44" ht="15.35" customHeight="1">
+      <c r="A44" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="B44">
+      <c r="B44" s="3">
         <v>3</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C44" t="s" s="2">
         <v>32</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D44" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E44" t="s">
+      <c r="E44" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="F44" t="s">
+      <c r="F44" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="G44" t="s">
+      <c r="G44" t="s" s="2">
         <v>60</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="s">
+    <row r="45" ht="15.35" customHeight="1">
+      <c r="A45" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="B45">
+      <c r="B45" s="3">
         <v>4</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C45" t="s" s="2">
         <v>33</v>
       </c>
-      <c r="D45" t="s">
+      <c r="D45" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E45" t="s">
+      <c r="E45" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="F45" t="s">
+      <c r="F45" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="G45" t="s">
+      <c r="G45" t="s" s="2">
         <v>60</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="s">
+    <row r="46" ht="15.35" customHeight="1">
+      <c r="A46" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="B46">
+      <c r="B46" s="3">
         <v>5</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C46" t="s" s="2">
         <v>36</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D46" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E46" t="s">
+      <c r="E46" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="F46" t="s">
+      <c r="F46" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="G46" t="s">
+      <c r="G46" t="s" s="2">
         <v>60</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="s">
+    <row r="47" ht="15.35" customHeight="1">
+      <c r="A47" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="B47">
+      <c r="B47" s="3">
         <v>6</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C47" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D47" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E47" t="s">
+      <c r="E47" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="F47" t="s">
+      <c r="F47" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="G47" t="s">
+      <c r="G47" t="s" s="2">
         <v>60</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="s">
+    <row r="48" ht="15.35" customHeight="1">
+      <c r="A48" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="B48">
+      <c r="B48" s="3">
         <v>7</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C48" t="s" s="2">
         <v>40</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D48" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E48" t="s">
+      <c r="E48" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="F48" t="s">
+      <c r="F48" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="G48" t="s">
+      <c r="G48" t="s" s="2">
         <v>60</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="s">
+    <row r="49" ht="15.35" customHeight="1">
+      <c r="A49" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="B49">
+      <c r="B49" s="3">
         <v>8</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C49" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="D49" t="s">
+      <c r="D49" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E49" t="s">
+      <c r="E49" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="F49" t="s">
+      <c r="F49" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="G49" t="s">
+      <c r="G49" t="s" s="2">
         <v>60</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="s">
+    <row r="50" ht="15.35" customHeight="1">
+      <c r="A50" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="B50">
+      <c r="B50" s="3">
         <v>9</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C50" t="s" s="2">
         <v>43</v>
       </c>
-      <c r="D50" t="s">
+      <c r="D50" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E50" t="s">
+      <c r="E50" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="F50" t="s">
+      <c r="F50" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="G50" t="s">
+      <c r="G50" t="s" s="2">
         <v>60</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="s">
+    <row r="51" ht="15.35" customHeight="1">
+      <c r="A51" t="s" s="2">
         <v>58</v>
       </c>
-      <c r="B51">
+      <c r="B51" s="3">
         <v>10</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C51" t="s" s="2">
         <v>46</v>
       </c>
-      <c r="D51" t="s">
+      <c r="D51" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E51" t="s">
+      <c r="E51" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="F51" t="s">
+      <c r="F51" t="s" s="2">
         <v>59</v>
       </c>
-      <c r="G51" t="s">
+      <c r="G51" t="s" s="2">
         <v>60</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="s">
+    <row r="52" ht="15.35" customHeight="1">
+      <c r="A52" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B52">
+      <c r="B52" s="3">
         <v>1</v>
       </c>
-      <c r="C52" t="s">
+      <c r="C52" t="s" s="2">
         <v>8</v>
       </c>
-      <c r="D52" t="s">
+      <c r="D52" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E52" t="s">
+      <c r="E52" t="s" s="2">
         <v>62</v>
       </c>
-      <c r="F52" t="s">
+      <c r="F52" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="G52" t="s">
+      <c r="G52" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="s">
+    <row r="53" ht="15.35" customHeight="1">
+      <c r="A53" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B53">
+      <c r="B53" s="3">
         <v>2</v>
       </c>
-      <c r="C53" t="s">
+      <c r="C53" t="s" s="2">
         <v>12</v>
       </c>
-      <c r="D53" t="s">
+      <c r="D53" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E53" t="s">
+      <c r="E53" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="F53" t="s">
+      <c r="F53" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="G53" t="s">
+      <c r="G53" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="s">
+    <row r="54" ht="15.35" customHeight="1">
+      <c r="A54" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B54">
+      <c r="B54" s="3">
         <v>3</v>
       </c>
-      <c r="C54" t="s">
+      <c r="C54" t="s" s="2">
         <v>15</v>
       </c>
-      <c r="D54" t="s">
+      <c r="D54" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E54" t="s">
+      <c r="E54" t="s" s="2">
         <v>65</v>
       </c>
-      <c r="F54" t="s">
+      <c r="F54" t="s" s="2">
         <v>66</v>
       </c>
-      <c r="G54" t="s">
+      <c r="G54" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="s">
+    <row r="55" ht="15.35" customHeight="1">
+      <c r="A55" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B55">
+      <c r="B55" s="3">
         <v>4</v>
       </c>
-      <c r="C55" t="s">
+      <c r="C55" t="s" s="2">
         <v>17</v>
       </c>
-      <c r="D55" t="s">
+      <c r="D55" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E55" t="s">
+      <c r="E55" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="F55" t="s">
+      <c r="F55" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="G55" t="s">
+      <c r="G55" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="s">
+    <row r="56" ht="15.35" customHeight="1">
+      <c r="A56" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B56">
+      <c r="B56" s="3">
         <v>5</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C56" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="D56" t="s">
+      <c r="D56" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E56" t="s">
+      <c r="E56" t="s" s="2">
         <v>62</v>
       </c>
-      <c r="F56" t="s">
+      <c r="F56" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="G56" t="s">
+      <c r="G56" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" t="s">
+    <row r="57" ht="15.35" customHeight="1">
+      <c r="A57" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B57">
+      <c r="B57" s="3">
         <v>6</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C57" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="D57" t="s">
+      <c r="D57" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E57" t="s">
+      <c r="E57" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="F57" t="s">
+      <c r="F57" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="G57" t="s">
+      <c r="G57" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" t="s">
+    <row r="58" ht="15.35" customHeight="1">
+      <c r="A58" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B58">
+      <c r="B58" s="3">
         <v>7</v>
       </c>
-      <c r="C58" t="s">
+      <c r="C58" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="D58" t="s">
+      <c r="D58" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E58" t="s">
+      <c r="E58" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="F58" t="s">
+      <c r="F58" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="G58" t="s">
+      <c r="G58" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="s">
+    <row r="59" ht="15.35" customHeight="1">
+      <c r="A59" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B59">
+      <c r="B59" s="3">
         <v>8</v>
       </c>
-      <c r="C59" t="s">
+      <c r="C59" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="D59" t="s">
+      <c r="D59" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E59" t="s">
+      <c r="E59" t="s" s="2">
         <v>65</v>
       </c>
-      <c r="F59" t="s">
+      <c r="F59" t="s" s="2">
         <v>66</v>
       </c>
-      <c r="G59" t="s">
+      <c r="G59" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="s">
+    <row r="60" ht="15.35" customHeight="1">
+      <c r="A60" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B60">
+      <c r="B60" s="3">
         <v>9</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C60" t="s" s="2">
         <v>27</v>
       </c>
-      <c r="D60" t="s">
+      <c r="D60" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E60" t="s">
+      <c r="E60" t="s" s="2">
         <v>67</v>
       </c>
-      <c r="F60" t="s">
+      <c r="F60" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="G60" t="s">
+      <c r="G60" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" t="s">
+    <row r="61" ht="15.35" customHeight="1">
+      <c r="A61" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B61">
+      <c r="B61" s="3">
         <v>10</v>
       </c>
-      <c r="C61" t="s">
+      <c r="C61" t="s" s="2">
         <v>28</v>
       </c>
-      <c r="D61" t="s">
+      <c r="D61" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E61" t="s">
+      <c r="E61" t="s" s="2">
         <v>67</v>
       </c>
-      <c r="F61" t="s">
+      <c r="F61" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="G61" t="s">
+      <c r="G61" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="s">
+    <row r="62" ht="15.35" customHeight="1">
+      <c r="A62" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B62">
+      <c r="B62" s="3">
         <v>11</v>
       </c>
-      <c r="C62" t="s">
+      <c r="C62" t="s" s="2">
         <v>29</v>
       </c>
-      <c r="D62" t="s">
+      <c r="D62" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E62" t="s">
+      <c r="E62" t="s" s="2">
         <v>67</v>
       </c>
-      <c r="F62" t="s">
+      <c r="F62" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="G62" t="s">
+      <c r="G62" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" t="s">
+    <row r="63" ht="15.35" customHeight="1">
+      <c r="A63" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B63">
+      <c r="B63" s="3">
         <v>12</v>
       </c>
-      <c r="C63" t="s">
+      <c r="C63" t="s" s="2">
         <v>31</v>
       </c>
-      <c r="D63" t="s">
+      <c r="D63" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E63" t="s">
+      <c r="E63" t="s" s="2">
         <v>62</v>
       </c>
-      <c r="F63" t="s">
+      <c r="F63" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="G63" t="s">
+      <c r="G63" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" t="s">
+    <row r="64" ht="15.35" customHeight="1">
+      <c r="A64" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B64">
+      <c r="B64" s="3">
         <v>13</v>
       </c>
-      <c r="C64" t="s">
+      <c r="C64" t="s" s="2">
         <v>32</v>
       </c>
-      <c r="D64" t="s">
+      <c r="D64" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E64" t="s">
+      <c r="E64" t="s" s="2">
         <v>62</v>
       </c>
-      <c r="F64" t="s">
+      <c r="F64" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="G64" t="s">
+      <c r="G64" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" t="s">
+    <row r="65" ht="15.35" customHeight="1">
+      <c r="A65" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B65">
+      <c r="B65" s="3">
         <v>14</v>
       </c>
-      <c r="C65" t="s">
+      <c r="C65" t="s" s="2">
         <v>33</v>
       </c>
-      <c r="D65" t="s">
+      <c r="D65" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E65" t="s">
+      <c r="E65" t="s" s="2">
         <v>65</v>
       </c>
-      <c r="F65" t="s">
+      <c r="F65" t="s" s="2">
         <v>66</v>
       </c>
-      <c r="G65" t="s">
+      <c r="G65" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" t="s">
+    <row r="66" ht="15.35" customHeight="1">
+      <c r="A66" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B66">
+      <c r="B66" s="3">
         <v>15</v>
       </c>
-      <c r="C66" t="s">
+      <c r="C66" t="s" s="2">
         <v>36</v>
       </c>
-      <c r="D66" t="s">
+      <c r="D66" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E66" t="s">
+      <c r="E66" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="F66" t="s">
+      <c r="F66" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="G66" t="s">
+      <c r="G66" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" t="s">
+    <row r="67" ht="15.35" customHeight="1">
+      <c r="A67" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B67">
+      <c r="B67" s="3">
         <v>16</v>
       </c>
-      <c r="C67" t="s">
+      <c r="C67" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="D67" t="s">
+      <c r="D67" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E67" t="s">
+      <c r="E67" t="s" s="2">
         <v>67</v>
       </c>
-      <c r="F67" t="s">
+      <c r="F67" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="G67" t="s">
+      <c r="G67" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" t="s">
+    <row r="68" ht="15.35" customHeight="1">
+      <c r="A68" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B68">
+      <c r="B68" s="3">
         <v>17</v>
       </c>
-      <c r="C68" t="s">
+      <c r="C68" t="s" s="2">
         <v>40</v>
       </c>
-      <c r="D68" t="s">
+      <c r="D68" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E68" t="s">
+      <c r="E68" t="s" s="2">
         <v>65</v>
       </c>
-      <c r="F68" t="s">
+      <c r="F68" t="s" s="2">
         <v>66</v>
       </c>
-      <c r="G68" t="s">
+      <c r="G68" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" t="s">
+    <row r="69" ht="15.35" customHeight="1">
+      <c r="A69" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B69">
+      <c r="B69" s="3">
         <v>18</v>
       </c>
-      <c r="C69" t="s">
+      <c r="C69" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="D69" t="s">
+      <c r="D69" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E69" t="s">
+      <c r="E69" t="s" s="2">
         <v>65</v>
       </c>
-      <c r="F69" t="s">
+      <c r="F69" t="s" s="2">
         <v>66</v>
       </c>
-      <c r="G69" t="s">
+      <c r="G69" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" t="s">
+    <row r="70" ht="15.35" customHeight="1">
+      <c r="A70" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B70">
+      <c r="B70" s="3">
         <v>19</v>
       </c>
-      <c r="C70" t="s">
+      <c r="C70" t="s" s="2">
         <v>43</v>
       </c>
-      <c r="D70" t="s">
+      <c r="D70" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E70" t="s">
+      <c r="E70" t="s" s="2">
         <v>62</v>
       </c>
-      <c r="F70" t="s">
+      <c r="F70" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="G70" t="s">
+      <c r="G70" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="s">
+    <row r="71" ht="15.35" customHeight="1">
+      <c r="A71" t="s" s="2">
         <v>61</v>
       </c>
-      <c r="B71">
+      <c r="B71" s="3">
         <v>20</v>
       </c>
-      <c r="C71" t="s">
+      <c r="C71" t="s" s="2">
         <v>46</v>
       </c>
-      <c r="D71" t="s">
+      <c r="D71" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E71" t="s">
+      <c r="E71" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="F71" t="s">
+      <c r="F71" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="G71" t="s">
+      <c r="G71" t="s" s="2">
         <v>64</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" t="s">
+    <row r="72" ht="15.35" customHeight="1">
+      <c r="A72" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B72">
+      <c r="B72" s="3">
         <v>1</v>
       </c>
-      <c r="C72" t="s">
+      <c r="C72" t="s" s="2">
         <v>8</v>
       </c>
-      <c r="D72" t="s">
+      <c r="D72" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E72" t="s">
+      <c r="E72" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F72" t="s">
+      <c r="F72" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G72" t="s">
+      <c r="G72" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" t="s">
+    <row r="73" ht="15.35" customHeight="1">
+      <c r="A73" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B73">
+      <c r="B73" s="3">
         <v>2</v>
       </c>
-      <c r="C73" t="s">
+      <c r="C73" t="s" s="2">
         <v>12</v>
       </c>
-      <c r="D73" t="s">
+      <c r="D73" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E73" t="s">
+      <c r="E73" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F73" t="s">
+      <c r="F73" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G73" t="s">
+      <c r="G73" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" t="s">
+    <row r="74" ht="15.35" customHeight="1">
+      <c r="A74" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B74">
+      <c r="B74" s="3">
         <v>3</v>
       </c>
-      <c r="C74" t="s">
+      <c r="C74" t="s" s="2">
         <v>15</v>
       </c>
-      <c r="D74" t="s">
+      <c r="D74" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E74" t="s">
+      <c r="E74" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F74" t="s">
+      <c r="F74" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G74" t="s">
+      <c r="G74" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" t="s">
+    <row r="75" ht="15.35" customHeight="1">
+      <c r="A75" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B75">
+      <c r="B75" s="3">
         <v>4</v>
       </c>
-      <c r="C75" t="s">
+      <c r="C75" t="s" s="2">
         <v>17</v>
       </c>
-      <c r="D75" t="s">
+      <c r="D75" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E75" t="s">
+      <c r="E75" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F75" t="s">
+      <c r="F75" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G75" t="s">
+      <c r="G75" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" t="s">
+    <row r="76" ht="15.35" customHeight="1">
+      <c r="A76" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B76">
+      <c r="B76" s="3">
         <v>5</v>
       </c>
-      <c r="C76" t="s">
+      <c r="C76" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="D76" t="s">
+      <c r="D76" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E76" t="s">
+      <c r="E76" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F76" t="s">
+      <c r="F76" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G76" t="s">
+      <c r="G76" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" t="s">
+    <row r="77" ht="15.35" customHeight="1">
+      <c r="A77" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B77">
+      <c r="B77" s="3">
         <v>6</v>
       </c>
-      <c r="C77" t="s">
+      <c r="C77" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="D77" t="s">
+      <c r="D77" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E77" t="s">
+      <c r="E77" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F77" t="s">
+      <c r="F77" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G77" t="s">
+      <c r="G77" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" t="s">
+    <row r="78" ht="15.35" customHeight="1">
+      <c r="A78" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B78">
+      <c r="B78" s="3">
         <v>7</v>
       </c>
-      <c r="C78" t="s">
+      <c r="C78" t="s" s="2">
         <v>23</v>
       </c>
-      <c r="D78" t="s">
+      <c r="D78" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E78" t="s">
+      <c r="E78" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F78" t="s">
+      <c r="F78" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G78" t="s">
+      <c r="G78" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" t="s">
+    <row r="79" ht="15.35" customHeight="1">
+      <c r="A79" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B79">
+      <c r="B79" s="3">
         <v>8</v>
       </c>
-      <c r="C79" t="s">
+      <c r="C79" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="D79" t="s">
+      <c r="D79" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E79" t="s">
+      <c r="E79" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F79" t="s">
+      <c r="F79" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G79" t="s">
+      <c r="G79" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" t="s">
+    <row r="80" ht="15.35" customHeight="1">
+      <c r="A80" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B80">
+      <c r="B80" s="3">
         <v>9</v>
       </c>
-      <c r="C80" t="s">
+      <c r="C80" t="s" s="2">
         <v>27</v>
       </c>
-      <c r="D80" t="s">
+      <c r="D80" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E80" t="s">
+      <c r="E80" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F80" t="s">
+      <c r="F80" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G80" t="s">
+      <c r="G80" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" t="s">
+    <row r="81" ht="15.35" customHeight="1">
+      <c r="A81" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B81">
+      <c r="B81" s="3">
         <v>10</v>
       </c>
-      <c r="C81" t="s">
+      <c r="C81" t="s" s="2">
         <v>28</v>
       </c>
-      <c r="D81" t="s">
+      <c r="D81" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E81" t="s">
+      <c r="E81" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F81" t="s">
+      <c r="F81" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G81" t="s">
+      <c r="G81" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" t="s">
+    <row r="82" ht="15.35" customHeight="1">
+      <c r="A82" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B82">
+      <c r="B82" s="3">
         <v>11</v>
       </c>
-      <c r="C82" t="s">
+      <c r="C82" t="s" s="2">
         <v>29</v>
       </c>
-      <c r="D82" t="s">
+      <c r="D82" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E82" t="s">
+      <c r="E82" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F82" t="s">
+      <c r="F82" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G82" t="s">
+      <c r="G82" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" t="s">
+    <row r="83" ht="15.35" customHeight="1">
+      <c r="A83" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B83">
+      <c r="B83" s="3">
         <v>12</v>
       </c>
-      <c r="C83" t="s">
+      <c r="C83" t="s" s="2">
         <v>31</v>
       </c>
-      <c r="D83" t="s">
+      <c r="D83" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E83" t="s">
+      <c r="E83" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F83" t="s">
+      <c r="F83" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G83" t="s">
+      <c r="G83" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" t="s">
+    <row r="84" ht="15.35" customHeight="1">
+      <c r="A84" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B84">
+      <c r="B84" s="3">
         <v>13</v>
       </c>
-      <c r="C84" t="s">
+      <c r="C84" t="s" s="2">
         <v>32</v>
       </c>
-      <c r="D84" t="s">
+      <c r="D84" t="s" s="2">
         <v>13</v>
       </c>
-      <c r="E84" t="s">
+      <c r="E84" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F84" t="s">
+      <c r="F84" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G84" t="s">
+      <c r="G84" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" t="s">
+    <row r="85" ht="15.35" customHeight="1">
+      <c r="A85" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B85">
+      <c r="B85" s="3">
         <v>14</v>
       </c>
-      <c r="C85" t="s">
+      <c r="C85" t="s" s="2">
         <v>33</v>
       </c>
-      <c r="D85" t="s">
+      <c r="D85" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E85" t="s">
+      <c r="E85" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F85" t="s">
+      <c r="F85" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G85" t="s">
+      <c r="G85" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" t="s">
+    <row r="86" ht="15.35" customHeight="1">
+      <c r="A86" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B86">
+      <c r="B86" s="3">
         <v>15</v>
       </c>
-      <c r="C86" t="s">
+      <c r="C86" t="s" s="2">
         <v>36</v>
       </c>
-      <c r="D86" t="s">
+      <c r="D86" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E86" t="s">
+      <c r="E86" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F86" t="s">
+      <c r="F86" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G86" t="s">
+      <c r="G86" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" t="s">
+    <row r="87" ht="15.35" customHeight="1">
+      <c r="A87" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B87">
+      <c r="B87" s="3">
         <v>16</v>
       </c>
-      <c r="C87" t="s">
+      <c r="C87" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="D87" t="s">
+      <c r="D87" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E87" t="s">
+      <c r="E87" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F87" t="s">
+      <c r="F87" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G87" t="s">
+      <c r="G87" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" t="s">
+    <row r="88" ht="15.35" customHeight="1">
+      <c r="A88" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B88">
+      <c r="B88" s="3">
         <v>17</v>
       </c>
-      <c r="C88" t="s">
+      <c r="C88" t="s" s="2">
         <v>40</v>
       </c>
-      <c r="D88" t="s">
+      <c r="D88" t="s" s="2">
         <v>16</v>
       </c>
-      <c r="E88" t="s">
+      <c r="E88" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F88" t="s">
+      <c r="F88" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G88" t="s">
+      <c r="G88" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" t="s">
+    <row r="89" ht="15.35" customHeight="1">
+      <c r="A89" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B89">
+      <c r="B89" s="3">
         <v>18</v>
       </c>
-      <c r="C89" t="s">
+      <c r="C89" t="s" s="2">
         <v>41</v>
       </c>
-      <c r="D89" t="s">
+      <c r="D89" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E89" t="s">
+      <c r="E89" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F89" t="s">
+      <c r="F89" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G89" t="s">
+      <c r="G89" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" t="s">
+    <row r="90" ht="15.35" customHeight="1">
+      <c r="A90" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B90">
+      <c r="B90" s="3">
         <v>19</v>
       </c>
-      <c r="C90" t="s">
+      <c r="C90" t="s" s="2">
         <v>43</v>
       </c>
-      <c r="D90" t="s">
+      <c r="D90" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E90" t="s">
+      <c r="E90" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F90" t="s">
+      <c r="F90" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G90" t="s">
+      <c r="G90" t="s" s="2">
         <v>71</v>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" t="s">
+    <row r="91" ht="15.35" customHeight="1">
+      <c r="A91" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="B91">
+      <c r="B91" s="3">
         <v>20</v>
       </c>
-      <c r="C91" t="s">
+      <c r="C91" t="s" s="2">
         <v>46</v>
       </c>
-      <c r="D91" t="s">
+      <c r="D91" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="E91" t="s">
+      <c r="E91" t="s" s="2">
         <v>69</v>
       </c>
-      <c r="F91" t="s">
+      <c r="F91" t="s" s="2">
         <v>70</v>
       </c>
-      <c r="G91" t="s">
+      <c r="G91" t="s" s="2">
         <v>71</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G91"/>
-  </ignoredErrors>
+  <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
+  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <headerFooter>
+    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>